<commit_message>
Refactor Excel file import methods to return lists of projects and plans; update main method to handle and display imported data
</commit_message>
<xml_diff>
--- a/.excel/projects.xlsx
+++ b/.excel/projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/one/IdeaProjects/cpiForecast/.excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC09967-8AB9-AC4E-995B-C67DBD75927F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E096B1B1-10F3-6C45-BA08-F2FFDDCF2259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5040" yWindow="1800" windowWidth="28300" windowHeight="17440" xr2:uid="{668DB8E8-A5D0-1E48-999F-BD4BCE261E1C}"/>
   </bookViews>
@@ -469,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -483,7 +483,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor Excel file import to handle null cells and update project data mapping; enhance main method to display imported projects
</commit_message>
<xml_diff>
--- a/.excel/projects.xlsx
+++ b/.excel/projects.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/one/IdeaProjects/cpiForecast/.excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E096B1B1-10F3-6C45-BA08-F2FFDDCF2259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3BA814-6748-6B4F-9555-F02B4E7A2FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="1800" windowWidth="28300" windowHeight="17440" xr2:uid="{668DB8E8-A5D0-1E48-999F-BD4BCE261E1C}"/>
+    <workbookView xWindow="5040" yWindow="1800" windowWidth="28300" windowHeight="17440" activeTab="1" xr2:uid="{668DB8E8-A5D0-1E48-999F-BD4BCE261E1C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="sample" sheetId="1" r:id="rId1"/>
+    <sheet name="TMS_Request List" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="6">
   <si>
     <t>改修プラン1(CPI1以上のサンプル)</t>
     <rPh sb="0" eb="2">
@@ -462,8 +463,8 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>789</v>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -483,6 +484,83 @@
         <v>1</v>
       </c>
       <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ED05485-CDD5-374A-B9BB-A9D89900FF2F}">
+  <dimension ref="H2:DC5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="8" max="8" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="5.28515625" customWidth="1"/>
+    <col min="12" max="12" width="30" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5" customWidth="1"/>
+    <col min="14" max="16" width="4.42578125" customWidth="1"/>
+    <col min="17" max="17" width="3.85546875" customWidth="1"/>
+    <col min="18" max="18" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="8:107">
+      <c r="H2">
+        <v>123</v>
+      </c>
+      <c r="L2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" t="s">
+        <v>1</v>
+      </c>
+      <c r="DC2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="8:107">
+      <c r="H3">
+        <v>456</v>
+      </c>
+      <c r="L3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P3" t="s">
+        <v>1</v>
+      </c>
+      <c r="DC3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="8:107">
+      <c r="H4">
+        <v>789</v>
+      </c>
+      <c r="L4" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" t="s">
+        <v>1</v>
+      </c>
+      <c r="DC4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="8:107">
+      <c r="H5" t="s">
+        <v>5</v>
+      </c>
+      <c r="L5" t="s">
+        <v>4</v>
+      </c>
+      <c r="P5" t="s">
+        <v>1</v>
+      </c>
+      <c r="DC5">
         <v>1</v>
       </c>
     </row>

</xml_diff>